<commit_message>
Cleaned up scap test content benchmark ID's
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="496" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28157E7D-8BFC-4FF8-9DBD-621605D420B7}"/>
+  <xr:revisionPtr revIDLastSave="514" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A0FB3F-62A5-425F-B7C5-68E76906E615}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" activeTab="2" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
+    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="SCAP 1.4 Self Assertion" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$J$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SCAP 1.4 Self Assertion'!$A$1:$J$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'SCAP 1.4 Self Assertion'!$A:$J</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="225">
   <si>
     <t>The product’s documentation (printed or electronic) MUST assert that it uses SCAP and its component specifications and explain relevant details to the users of the product.</t>
   </si>
@@ -740,6 +740,162 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>SCAP.T.2000.1: The tester SHALL run the product using a valid SCAP data stream against the target systems of the target platform type. 
+SCAP.T.2000.2: The tester SHALL validate the resulting SCAP data stream by importing it into the SCAPVal utility and checking for any validation errors.
+SCAP.T.2000.3: The tester SHALL validate that the resulting SCAP data stream is available for viewing by the user.
+SCAP.T.2000.4: The tester SHALL capture the successful results of the import and verify the correctness of the results.</t>
+  </si>
+  <si>
+    <t>SCAP.T.2200.1: The tester SHALL run the product using valid SCAP data stream files against the target systems of the target platform type. 
+SCAP.T.2200.2: The tester SHALL validate the resulting SCAP data stream by importing it into the SCAPVal utility and checking for any validation errors.
+SCAP.T.2200.3: The tester SHALL validate that the resulting SCAP data stream is available for viewing by the user.</t>
+  </si>
+  <si>
+    <t>Use any applicable content from SCAP_Test_Content\R700</t>
+  </si>
+  <si>
+    <t>Use content from SCAP_Test_Content\R2200</t>
+  </si>
+  <si>
+    <t>Use content from SCAP_Test_Content\R2100
+questionnaire_results:
+  ocil:validation_program:questionnaire:1" result="FAIL"
+  ocil:validation_program:questionnaire:2" result="PASS"
+  ocil:validation_program:questionnaire:3" result="PASS"</t>
+  </si>
+  <si>
+    <t>1.  Install and run any single SCAP 1.4 content stream that is supported by the SCAP interpreter in the R700 directory
+2.  Select a profile a perform a scan
+3.  Perform scans, ensuring that XML results are schema valid.
+4.  No errors are reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.  Install r500-datastream.xml
+2.  Select either of the two source datastreams contained in the r500 datastream collection.
+3.  Perform a scan
+4.  Select the other data stream in the r500 datastream collection
+5.  Tool can display multiple datastreams in a collection, and no errors are reported when performing scans.
+</t>
+  </si>
+  <si>
+    <t>1.  Install U_MS_Defender_Antivirus_V2R7_STIG_SCAP_1-4_Benchmark-enhancedV13-signed.zip
+a.  Content should install and scans possible with a valid XML digital signature
+2.  Install U_MS_Edge_V2R4_STIG_SCAP_1-4_Benchmark-enhancedV14-corrupt.zip
+a.  Scanner should report that the XML digital signature validation failed, and refuse to perform a scan.</t>
+  </si>
+  <si>
+    <t>SCAP.T.1000.1:   User the vendor product, the tester SHALL attempt to install and execute a SCAP source datastream that has been signed by a private/untrusted  digital certificate.</t>
+  </si>
+  <si>
+    <t>Refer to vendor documentation</t>
+  </si>
+  <si>
+    <t>The product shall include ident system information (CCE, CVE, CCI, etc. ) from the XCCDF rule as part of the xccdf rule-result</t>
+  </si>
+  <si>
+    <t>Invalid content for testing the SCAP.R.400 requirement
+- r400.2.1-datastream.xml - invalid according to the XML schema representation for the source data stream
+- r400.2.2-datastream.xml - Not well formed XML content
+- r400.2.3-datastream.xml - invalid according to the Schematron schema representation for the source data stream
+Optional:  Compare errors reported from the vendor product to those reported in the ValidationFiles directory.  Errors should be similar</t>
+  </si>
+  <si>
+    <t>Invalid content for testing the SCAP.R.400 requirement
+- r1300.2.2-xccdf-schematron-errors.xml - invalid according to the Schematron schema representation for the source data stream (XCCDF)
+- r1300.3.1-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (OVAL)
+- r1300.3.2-oval-schematron-errors.xml - invalid according to the Schematron schema representation for the source data stream (OVAL)
+- r1300.3.3-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (OVAL namespace)
+- r1300.4.1-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (CPE Dictionary)</t>
+  </si>
+  <si>
+    <t>1.  Install and run any single SCAP 1.4 content stream from the \SCAP_Test_Content\R1500 directory that is supported by the SCAP interpreter from R700
+2.  Select a profile a perform a scan
+3.  Perform scans, ensuring that XML results are schema valid.
+4.  No errors are reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.  Install oval-def-ext.zip from the SCAP_Test_Content\R1900 directory.    This should install both the OVAL content file and the OVAL Variables XML file into the product.   If after performing a scan, the product cannot locate the OVAL Variables file, refer to product documentation on how to install external variables XML files.
+2.  Scan any target with the oval-def-ext content enabled, oval definition and all tests should return true if the product supports external variables.
+</t>
+  </si>
+  <si>
+    <t>1.  Install and run all content that the SCAP interpreter under test supports from SCAP_Test_Content\R1100
+2.  Perform scans, ensuring that XML results are schema valid.
+3.  No errors are reported.</t>
+  </si>
+  <si>
+    <t>SCAP 1.3 Compatiblity</t>
+  </si>
+  <si>
+    <t>SCAP.T.4100.1: The tester SHALL import the SCAP 1.4 source data stream, apply it to a known target, and produce an SCAP result data stream conforming to the ARF specification.
+SCAP.T.4100.2: The tester SHALL validate the results produced using SCAPVal; the validation MUST NOT produce any errors.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\windows.
+3.  Scan Windows targets with all OVAL content from steps 1-2, and review results.
+All definitions should return 'true' unless specifically stated in the definition title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\linux.
+3.  Install all OVAL content from OVAL_Test_Content\unix.
+4.  Scan Linux targets with all OVAL content from steps 1-3, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\macos.
+3.  Scan macOS targets with all OVAL content from steps 1-2, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
+2.  Install all OVAL content from OVAL_Test_Content\solaris.
+3.  Install all OVAL content from OVAL_Test_Content\unix.
+4.  Scan Solaris targets with all OVAL content from steps 1-3, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\ios.
+2.  Scan cisco targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t>1.  Install all OVAL content from OVAL_Test_Content\ios-xe.
+2.  Scan cisco-xe targets with all OVAL content from step 1, and review results.
+All defintions should return 'true' unless specficially stated in the defintion title.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SCAP 1.3 backward compatibility </t>
+  </si>
+  <si>
+    <t>Test Procedures</t>
+  </si>
+  <si>
+    <t>1.  Install the R1000_signed_by_untrusted_private_cert.xml from in the R1000 directory.  This file is from NIST's SCAP 1.3 validation program, but has been digitally signed by a self signed cert that should not be (by default) trusted by any vendor product.
+2.  Attempt to have the product validate the digital certificate by vendor documentation, and document the errors, likely that the certificate chain could not be verified.
+Note 1:  If the content does pass digital signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verify, and then retest.</t>
+  </si>
+  <si>
+    <t>SCAP.R.4500</t>
+  </si>
+  <si>
+    <t>SCAP.V.4500.1:  The vendor shall provide documentation on how it creates human readable results from OVAL/OCIL and saves them to XCCDF rule-results message elemnt with severity of 'info'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCAP.T.4500.1:  The tester SHALL review the XCCDF rule results and confirm that the xccdf rule-result message exists with a severity of 'info'.  The contents of this element are at the discretion of the vendor, but should provide sufficient information from OVAL/OCIL to know why the rule passed or failed. </t>
+  </si>
+  <si>
+    <t>1.  Review a sample of XCCDF results from R700 and view XCCDF results to ensure that each rule-result contains a message with severity='info' and the data it contains is sufficient to understand why the rule passed or failed.</t>
+  </si>
+  <si>
+    <t>The product shall include human readable results from OVAL/OCIL as part of XCCDF rule-results.</t>
+  </si>
+  <si>
+    <t>1.0 Release Candidate 1 (May 15, 2026)</t>
   </si>
   <si>
     <r>
@@ -795,151 +951,14 @@
    c.  Select Pass/Fail or Not Applicable for the Result.
 3.  Zip up all test content results (XML, HTML, Text etc..) 
 4.  Create a SCAP 1.4 Implentation Statement (Saved to a PDF)
-5.  Send Self Assertion bundle to (????)
-    a.  This completed spreadsheet
-    b.  SCAP 1.4 Implementaton Statement (PDF Format)
-    c.  Zipped archive of all tests results
-    d. Vendor or Application Logo ( 300 x 300 square in PNG Format)
+5.  Commit results to github in a new directory based on your Vendor Name
+    a.  https://github.com/OVAL-Community/SCAP-Self-Assertion/tree/main/SCAP_1.4/Completed_Self_Assertions/&lt;Vendor Name&gt;
+    b.  This completed spreadsheet
+    c.  SCAP 1.4 Implementaton Statement (PDF Format)
+    d.  Vendor or Application Logo ( 300 x 300 square in PNG Format)
+    e.  Sub-Directory of test results from SCAP and OVAL test content.  
 </t>
     </r>
-  </si>
-  <si>
-    <t>SCAP.T.2000.1: The tester SHALL run the product using a valid SCAP data stream against the target systems of the target platform type. 
-SCAP.T.2000.2: The tester SHALL validate the resulting SCAP data stream by importing it into the SCAPVal utility and checking for any validation errors.
-SCAP.T.2000.3: The tester SHALL validate that the resulting SCAP data stream is available for viewing by the user.
-SCAP.T.2000.4: The tester SHALL capture the successful results of the import and verify the correctness of the results.</t>
-  </si>
-  <si>
-    <t>SCAP.T.2200.1: The tester SHALL run the product using valid SCAP data stream files against the target systems of the target platform type. 
-SCAP.T.2200.2: The tester SHALL validate the resulting SCAP data stream by importing it into the SCAPVal utility and checking for any validation errors.
-SCAP.T.2200.3: The tester SHALL validate that the resulting SCAP data stream is available for viewing by the user.</t>
-  </si>
-  <si>
-    <t>Use any applicable content from SCAP_Test_Content\R700</t>
-  </si>
-  <si>
-    <t>Use content from SCAP_Test_Content\R2200</t>
-  </si>
-  <si>
-    <t>Use content from SCAP_Test_Content\R2100
-questionnaire_results:
-  ocil:validation_program:questionnaire:1" result="FAIL"
-  ocil:validation_program:questionnaire:2" result="PASS"
-  ocil:validation_program:questionnaire:3" result="PASS"</t>
-  </si>
-  <si>
-    <t>1.  Install and run any single SCAP 1.4 content stream that is supported by the SCAP interpreter in the R700 directory
-2.  Select a profile a perform a scan
-3.  Perform scans, ensuring that XML results are schema valid.
-4.  No errors are reported.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.  Install r500-datastream.xml
-2.  Select either of the two source datastreams contained in the r500 datastream collection.
-3.  Perform a scan
-4.  Select the other data stream in the r500 datastream collection
-5.  Tool can display multiple datastreams in a collection, and no errors are reported when performing scans.
-</t>
-  </si>
-  <si>
-    <t>1.  Install U_MS_Defender_Antivirus_V2R7_STIG_SCAP_1-4_Benchmark-enhancedV13-signed.zip
-a.  Content should install and scans possible with a valid XML digital signature
-2.  Install U_MS_Edge_V2R4_STIG_SCAP_1-4_Benchmark-enhancedV14-corrupt.zip
-a.  Scanner should report that the XML digital signature validation failed, and refuse to perform a scan.</t>
-  </si>
-  <si>
-    <t>SCAP.T.1000.1:   User the vendor product, the tester SHALL attempt to install and execute a SCAP source datastream that has been signed by a private/untrusted  digital certificate.</t>
-  </si>
-  <si>
-    <t>Refer to vendor documentation</t>
-  </si>
-  <si>
-    <t>The product shall include ident system information (CCE, CVE, CCI, etc. ) from the XCCDF rule as part of the xccdf rule-result</t>
-  </si>
-  <si>
-    <t>Invalid content for testing the SCAP.R.400 requirement
-- r400.2.1-datastream.xml - invalid according to the XML schema representation for the source data stream
-- r400.2.2-datastream.xml - Not well formed XML content
-- r400.2.3-datastream.xml - invalid according to the Schematron schema representation for the source data stream
-Optional:  Compare errors reported from the vendor product to those reported in the ValidationFiles directory.  Errors should be similar</t>
-  </si>
-  <si>
-    <t>Invalid content for testing the SCAP.R.400 requirement
-- r1300.2.2-xccdf-schematron-errors.xml - invalid according to the Schematron schema representation for the source data stream (XCCDF)
-- r1300.3.1-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (OVAL)
-- r1300.3.2-oval-schematron-errors.xml - invalid according to the Schematron schema representation for the source data stream (OVAL)
-- r1300.3.3-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (OVAL namespace)
-- r1300.4.1-oval-schema-errors.xml - invalid according to the XML schema representation for the source data stream (CPE Dictionary)</t>
-  </si>
-  <si>
-    <t>1.  Install and run any single SCAP 1.4 content stream from the \SCAP_Test_Content\R1500 directory that is supported by the SCAP interpreter from R700
-2.  Select a profile a perform a scan
-3.  Perform scans, ensuring that XML results are schema valid.
-4.  No errors are reported.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.  Install oval-def-ext.zip from the SCAP_Test_Content\R1900 directory.    This should install both the OVAL content file and the OVAL Variables XML file into the product.   If after performing a scan, the product cannot locate the OVAL Variables file, refer to product documentation on how to install external variables XML files.
-2.  Scan any target with the oval-def-ext content enabled, oval definition and all tests should return true if the product supports external variables.
-</t>
-  </si>
-  <si>
-    <t>1.  Install and run all content that the SCAP interpreter under test supports from SCAP_Test_Content\R1100
-2.  Perform scans, ensuring that XML results are schema valid.
-3.  No errors are reported.</t>
-  </si>
-  <si>
-    <t>SCAP 1.3 Compatiblity</t>
-  </si>
-  <si>
-    <t>SCAP.T.4100.1: The tester SHALL import the SCAP 1.4 source data stream, apply it to a known target, and produce an SCAP result data stream conforming to the ARF specification.
-SCAP.T.4100.2: The tester SHALL validate the results produced using SCAPVal; the validation MUST NOT produce any errors.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
-2.  Install all OVAL content from OVAL_Test_Content\windows.
-3.  Scan Windows targets with all OVAL content from steps 1-2, and review results.
-All definitions should return 'true' unless specifically stated in the definition title.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
-2.  Install all OVAL content from OVAL_Test_Content\linux.
-3.  Install all OVAL content from OVAL_Test_Content\unix.
-4.  Scan Linux targets with all OVAL content from steps 1-3, and review results.
-All defintions should return 'true' unless specficially stated in the defintion title.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
-2.  Install all OVAL content from OVAL_Test_Content\macos.
-3.  Scan macOS targets with all OVAL content from steps 1-2, and review results.
-All defintions should return 'true' unless specficially stated in the defintion title.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\agnostic.
-2.  Install all OVAL content from OVAL_Test_Content\solaris.
-3.  Install all OVAL content from OVAL_Test_Content\unix.
-4.  Scan Solaris targets with all OVAL content from steps 1-3, and review results.
-All defintions should return 'true' unless specficially stated in the defintion title.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\ios.
-2.  Scan cisco targets with all OVAL content from step 1, and review results.
-All defintions should return 'true' unless specficially stated in the defintion title.</t>
-  </si>
-  <si>
-    <t>1.  Install all OVAL content from OVAL_Test_Content\ios-xe.
-2.  Scan cisco-xe targets with all OVAL content from step 1, and review results.
-All defintions should return 'true' unless specficially stated in the defintion title.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> SCAP 1.3 backward compatibility </t>
-  </si>
-  <si>
-    <t>Test Procedures</t>
-  </si>
-  <si>
-    <t>1.  Install the R1000_signed_by_untrusted_private_cert.xml from in the R1000 directory.  This file is from NIST's SCAP 1.3 validation program, but has been digitally signed by a self signed cert that should not be (by default) trusted by any vendor product.
-2.  Attempt to have the product validate the digital certificate by vendor documentation, and document the errors, likely that the certificate chain could not be verified.
-Note 1:  If the content does pass digital signature validation, determine where the trusted certificate store is located, and remove the certificates that are used to verify, and then retest.</t>
   </si>
 </sst>
 </file>
@@ -1105,10 +1124,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1442,7 +1457,7 @@
     </row>
     <row r="2" spans="1:1" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>191</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -1512,7 +1527,9 @@
       <c r="A8" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="14" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
@@ -1534,7 +1551,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B12" s="14"/>
     </row>
@@ -1549,7 +1566,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S42"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" style="10" customWidth="1"/>
@@ -1572,7 +1589,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
@@ -1587,7 +1604,7 @@
         <v>169</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>20</v>
@@ -1699,7 +1716,7 @@
         <v>19</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
@@ -1723,7 +1740,7 @@
         <v>18</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
@@ -1771,7 +1788,7 @@
         <v>29</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
@@ -1819,7 +1836,7 @@
         <v>35</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -1840,10 +1857,10 @@
         <v>180</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
@@ -1869,7 +1886,7 @@
         <v>40</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
@@ -1917,7 +1934,7 @@
         <v>46</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
@@ -1963,7 +1980,7 @@
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
@@ -1987,7 +2004,7 @@
         <v>66</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -2008,10 +2025,10 @@
         <v>68</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
@@ -2035,7 +2052,7 @@
         <v>72</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
@@ -2056,10 +2073,10 @@
         <v>75</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
@@ -2081,7 +2098,7 @@
         <v>78</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
@@ -2105,7 +2122,7 @@
         <v>86</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
@@ -2177,7 +2194,7 @@
         <v>98</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
@@ -2249,7 +2266,7 @@
         <v>113</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
@@ -2297,7 +2314,7 @@
         <v>122</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -2321,7 +2338,7 @@
         <v>126</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
@@ -2345,7 +2362,7 @@
         <v>130</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
@@ -2366,32 +2383,34 @@
         <v>133</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
+    <row r="34" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="5" t="s">
-        <v>181</v>
+        <v>218</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>186</v>
+        <v>219</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>183</v>
+        <v>220</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
@@ -2401,41 +2420,41 @@
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>184</v>
+        <v>201</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
     </row>
-    <row r="36" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="5" t="s">
-        <v>135</v>
+        <v>182</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>153</v>
+        <v>187</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
@@ -2445,85 +2464,85 @@
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
     </row>
-    <row r="38" spans="1:10" ht="102" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
     </row>
-    <row r="39" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ht="102" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
     </row>
-    <row r="40" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
@@ -2533,27 +2552,49 @@
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
     </row>
+    <row r="42" spans="1:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J41" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}"/>
+  <autoFilter ref="A1:J42" xr:uid="{B5C7E2F8-1D87-4E2E-8196-7F95EBE1FA6F}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I41" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I42" xr:uid="{1C488EE4-4AD3-49DB-8EC8-8A5BD2F07EE9}">
       <formula1>$S$1:$S$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Updated sample results to be non-zipped per OVAL board.  Updated checklist to include new XCCDF rule-result requirement
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flankspeed-my.sharepoint-mil.us/personal/jack_r_vanderpol_civ_us_navy_mil/Documents/Documents/github/SCAP-Self-Assertion/SCAP_1.4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="514" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9A0FB3F-62A5-425F-B7C5-68E76906E615}"/>
+  <xr:revisionPtr revIDLastSave="515" documentId="8_{E8FF32BF-741C-48F8-A195-54C03221DD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91971601-D4C5-4D7A-811F-2896530FDE45}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{91EDF8AA-12A4-463E-9EF6-D256E525D567}"/>
   </bookViews>
@@ -956,7 +956,7 @@
     b.  This completed spreadsheet
     c.  SCAP 1.4 Implementaton Statement (PDF Format)
     d.  Vendor or Application Logo ( 300 x 300 square in PNG Format)
-    e.  Sub-Directory of test results from SCAP and OVAL test content.  
+    e.  Sub-Directory of test results from SCAP and OVAL test content, including ARF, XCCDF and OVAL results.
 </t>
     </r>
   </si>
@@ -1124,6 +1124,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Fixed a couple tab/space issues with readme data
</commit_message>
<xml_diff>
--- a/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
+++ b/SCAP_1.4/SCAP_1.4_Self_Assertion_Checklist.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId3"/>
@@ -66,16 +66,16 @@
 1.  Fill out the Vendor Information tab
 2.  Fill out the OVAL Test Declarations tab
 3.  Complete the SCAP 1.4 Self Assertion tab
-   a.  Follow the Test Procedures and Detailed Test Instructions.
-   b.  Fill in the Detailed Results text entry field:  Document the result of the test with a human readable synopsis of the test results.  
-   c.  Select Pass/Fail or Not Applicable for the result.
+	a.  Follow the Test Procedures and Detailed Test Instructions.
+	b.  Fill in the Detailed Results text entry field:  Document the result of the test with a human readable synopsis of the test results.  
+	c.  Select Pass/Fail or Not Applicable for the result.
 4.  Create a SCAP 1.4 Implementation Statement (Saved to a PDF)
 5.  Commit results to github in a new directory based on your Vendor Name
-    a.  https://github.com/OVAL-Community/SCAP-Self-Assertion/tree/main/SCAP_1.4/Completed_Self_Assertions/&lt;Vendor Name&gt;.
-    b.  This completed spreadsheet.
-    c.  SCAP 1.4 Implementation Statement (PDF Format).
-    d.  Vendor or Application Logo (300 x 300 square in PNG Format).
-    e.  Sub-Directory of test results from SCAP and OVAL test content, including ARF, XCCDF and OVAL results.
+	a.  https://github.com/OVAL-Community/SCAP-Self-Assertion/tree/main/SCAP_1.4/Completed_Self_Assertions/&lt;Vendor Name&gt;.
+	b.  This completed spreadsheet.
+	c.  SCAP 1.4 Implementation Statement (PDF Format).
+	d.  Vendor or Application Logo (300 x 300 square in PNG Format).
+	e.  Sub-Directory of test results from SCAP and OVAL test content, including ARF, XCCDF and OVAL results.
 </t>
   </si>
   <si>

</xml_diff>